<commit_message>
set up simple gui
</commit_message>
<xml_diff>
--- a/vesicles/directories.xlsx
+++ b/vesicles/directories.xlsx
@@ -1,64 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/jkerssemakers_tudelft_nl/Documents/Documents/GitHub/CD23_vesicles/vesicles/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_2B59D2BFD370DBDA4F331C104C1510344D078DFF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C5D1BE5-DC7C-4849-A598-D0C48E136E69}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>experiment_path_in</t>
-  </si>
-  <si>
-    <t>experiment_path_out</t>
-  </si>
-  <si>
-    <t>experiment_use_it</t>
-  </si>
-  <si>
-    <t>remarks</t>
-  </si>
-  <si>
-    <t>M:\tnw\bn\cd\Shared\Jacob\TESTdata_in\2025_Charu\pilots\20082025_CS_test</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -66,26 +45,94 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -373,36 +420,47 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="25.81640625" customWidth="1"/>
-    <col min="3" max="4" width="16" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>experiment_path_in</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>experiment_path_out</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>experiment_use_it</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>M:\tnw\bn\cd\Shared\Jacob\TESTdata_in\2025_Charu\pilots\20082025_CS_test</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
setting up GUI based UI_XLS
</commit_message>
<xml_diff>
--- a/vesicles/directories.xlsx
+++ b/vesicles/directories.xlsx
@@ -1,43 +1,67 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/jkerssemakers_tudelft_nl/Documents/Documents/GitHub/CD23_vesicles/vesicles/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_2B59D2BFD360DC7675EBDF905C1510344D078DEF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9801975-0ED1-4074-B1FB-F14DC4372F3E}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="7845" yWindow="195" windowWidth="20580" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+  <si>
+    <t>experiment_path_in</t>
+  </si>
+  <si>
+    <t>experiment_path_out</t>
+  </si>
+  <si>
+    <t>experiment_use_it</t>
+  </si>
+  <si>
+    <t>remarks</t>
+  </si>
+  <si>
+    <t>any_directory\any_sub_directory</t>
+  </si>
+  <si>
+    <t>tadaaaa</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,94 +69,26 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,47 +376,41 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="32.7109375" customWidth="1"/>
+    <col min="2" max="4" width="25.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>experiment_path_in</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>experiment_path_out</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>experiment_use_it</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>remarks</t>
-        </is>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>M:\tnw\bn\cd\Shared\Jacob\TESTdata_in\2025_Charu\pilots\20082025_CS_test</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="n">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
setting up db-excel interaction
</commit_message>
<xml_diff>
--- a/vesicles/directories.xlsx
+++ b/vesicles/directories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/jkerssemakers_tudelft_nl/Documents/Documents/GitHub/CD23_vesicles/vesicles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_2B59D2BFD360DC7675EBDF905C1510344D078DEF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9801975-0ED1-4074-B1FB-F14DC4372F3E}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_2B59D2BFD3B0DC3526FB0593561510344D078D05" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4498431C-A606-4EF5-9B05-6C04DD6127C9}"/>
   <bookViews>
     <workbookView xWindow="7845" yWindow="195" windowWidth="20580" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+  <si>
+    <t>experiment_id</t>
+  </si>
   <si>
     <t>experiment_path_in</t>
   </si>
@@ -377,14 +380,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.7109375" customWidth="1"/>
-    <col min="2" max="4" width="25.28515625" customWidth="1"/>
+    <col min="1" max="5" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -397,19 +399,22 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>4</v>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>-1</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
-        <v>3</v>
+      <c r="E2" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>